<commit_message>
Update report pipeline documentation and outputs
</commit_message>
<xml_diff>
--- a/OECD-Reports/V4-formatted-Data Points Graphs_Italy (1).xlsx
+++ b/OECD-Reports/V4-formatted-Data Points Graphs_Italy (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wjproject.sharepoint.com/research/Programmatic/Data Analytics/6. Country Reports/OECD-EULNS/OECD-Reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="271" documentId="13_ncr:1_{72F0734B-92D2-47E2-9DC9-09469FE5BF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA965718-E85C-5C4D-B1F5-493B96B3D982}"/>
+  <xr:revisionPtr revIDLastSave="389" documentId="13_ncr:1_{72F0734B-92D2-47E2-9DC9-09469FE5BF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF403894-14C8-C14F-AC35-712D84C48BE5}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="13" xr2:uid="{352B6E54-51F9-45EB-BD81-34DAE6470495}"/>
+    <workbookView xWindow="-49000" yWindow="-10340" windowWidth="19300" windowHeight="20120" firstSheet="8" activeTab="16" xr2:uid="{352B6E54-51F9-45EB-BD81-34DAE6470495}"/>
   </bookViews>
   <sheets>
     <sheet name="General info" sheetId="96" r:id="rId1"/>
@@ -103,7 +103,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="108">
   <si>
     <t>Category</t>
   </si>
@@ -433,11 +433,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -567,9 +565,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -583,6 +579,10 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -774,7 +774,7 @@
                   <c:v>0.314</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.26700000000000002</c:v>
+                  <c:v>0.26</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0.23400000000000001</c:v>
@@ -14831,22 +14831,22 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0.51</c:v>
+                  <c:v>0.59</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.58799999999999997</c:v>
+                  <c:v>0.65</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>0.59</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>0.6</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.60099999999999998</c:v>
-                </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.66</c:v>
+                  <c:v>0.59</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.60099999999999998</c:v>
+                  <c:v>0.51</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -16189,7 +16189,7 @@
                   <c:v>0.53</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.72</c:v>
+                  <c:v>0.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -17219,7 +17219,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>  4.0 </a:t>
+                      <a:t>  3.7 </a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -17271,7 +17271,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>  4.2 </a:t>
+                      <a:t>  3.9 </a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -17364,11 +17364,11 @@
               <c:numCache>
                 <c:formatCode>_-* #,##0.0_-;\-* #,##0.0_-;_-* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-">
-                  <c:v>4</c:v>
+                <c:pt idx="0">
+                  <c:v>3.7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.2</c:v>
+                  <c:v>3.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -17465,10 +17465,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -18012,7 +18012,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>5.3</a:t>
+                      <a:t>5.0</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -18031,6 +18031,7 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:showDataLabelsRange val="0"/>
@@ -18064,7 +18065,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>5.3</a:t>
+                      <a:t>4.6</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -18083,6 +18084,7 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:showDataLabelsRange val="0"/>
@@ -18094,58 +18096,6 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="2"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
-                    <a:spAutoFit/>
-                  </a:bodyPr>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr>
-                      <a:defRPr sz="700" b="0" i="0">
-                        <a:solidFill>
-                          <a:schemeClr val="bg1"/>
-                        </a:solidFill>
-                        <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
-                      </a:defRPr>
-                    </a:pPr>
-                    <a:r>
-                      <a:rPr lang="en-US" sz="700" b="0" i="0">
-                        <a:solidFill>
-                          <a:schemeClr val="bg1"/>
-                        </a:solidFill>
-                        <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <a:t>4.8</a:t>
-                    </a:r>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:dLblPos val="ctr"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:showDataLabelsRange val="0"/>
-                </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000002-7868-4252-B8FC-AF08EC101490}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="3"/>
               <c:tx>
                 <c:rich>
                   <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
@@ -18187,6 +18137,60 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:showDataLabelsRange val="0"/>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-7868-4252-B8FC-AF08EC101490}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                    <a:spAutoFit/>
+                  </a:bodyPr>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="700" b="0" i="0">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                        <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" sz="700" b="0" i="0">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                        <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <a:t>4.0</a:t>
+                    </a:r>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:dLblPos val="ctr"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:showDataLabelsRange val="0"/>
@@ -18220,7 +18224,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>3.3</a:t>
+                      <a:t>3.2</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -18239,6 +18243,7 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:showDataLabelsRange val="0"/>
@@ -18272,7 +18277,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>3.1</a:t>
+                      <a:t>3.0</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -18291,6 +18296,7 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:showDataLabelsRange val="0"/>
@@ -18330,6 +18336,7 @@
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
+            <c:separator>, </c:separator>
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -18374,25 +18381,25 @@
             <c:numRef>
               <c:f>'g1-3'!$D$23:$D$28</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>_-* #,##0.0_-;\-* #,##0.0_-;_-* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>5.3</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.3</c:v>
+                  <c:v>4.5999999999999996</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.8</c:v>
+                  <c:v>4.4000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.4000000000000004</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.3</c:v>
+                  <c:v>3.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.1</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -18500,22 +18507,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -19216,7 +19223,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>3.4</a:t>
+                      <a:t>3.3</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -19268,7 +19275,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>5.7</a:t>
+                      <a:t>5.0</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -19359,13 +19366,13 @@
             <c:numRef>
               <c:f>'g1-3'!$D$30:$D$31</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
+                <c:formatCode>_-* #,##0.0_-;\-* #,##0.0_-;_-* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>3.4</c:v>
+                  <c:v>3.3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.7</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -19458,13 +19465,13 @@
             <c:numRef>
               <c:f>'g1-3'!$E$30:$E$31</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -19917,7 +19924,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>4.1</a:t>
+                      <a:t>3.8</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -19936,6 +19943,7 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:showDataLabelsRange val="0"/>
@@ -19969,7 +19977,7 @@
                         </a:solidFill>
                         <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <a:t>4.2</a:t>
+                      <a:t>4.0</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -19988,6 +19996,7 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
+              <c:separator>, </c:separator>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:showDataLabelsRange val="0"/>
@@ -20028,6 +20037,7 @@
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
+            <c:separator>, </c:separator>
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -20060,13 +20070,13 @@
             <c:numRef>
               <c:f>'g1-3'!$D$33:$D$34</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>_-* #,##0.0_-;\-* #,##0.0_-;_-* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.2</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -20162,10 +20172,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0999999999999996</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -22734,15 +22744,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>594033</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>149327</xdr:rowOff>
+      <xdr:colOff>737420</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>5940</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>519266</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>92177</xdr:rowOff>
+      <xdr:colOff>662653</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>143387</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -22777,13 +22787,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615167</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>36164</xdr:rowOff>
+      <xdr:rowOff>62901</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615167</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>37427</xdr:rowOff>
+      <xdr:rowOff>64164</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -22800,7 +22810,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1615167" y="36164"/>
+          <a:off x="1615167" y="62901"/>
           <a:ext cx="0" cy="5616000"/>
         </a:xfrm>
         <a:prstGeom prst="line">
@@ -22833,15 +22843,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>483220</xdr:colOff>
+      <xdr:colOff>376274</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>113814</xdr:rowOff>
+      <xdr:rowOff>140551</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>483220</xdr:colOff>
+      <xdr:colOff>376274</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>115077</xdr:rowOff>
+      <xdr:rowOff>141814</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -22858,7 +22868,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6151431" y="113814"/>
+          <a:off x="6044485" y="140551"/>
           <a:ext cx="0" cy="5616000"/>
         </a:xfrm>
         <a:prstGeom prst="line">
@@ -22893,13 +22903,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>54452</xdr:rowOff>
+      <xdr:rowOff>81189</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615168</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>77753</xdr:rowOff>
+      <xdr:rowOff>104490</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -22914,7 +22924,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="54452"/>
+          <a:off x="0" y="81189"/>
           <a:ext cx="1615168" cy="584775"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -23042,13 +23052,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>175167</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>13554</xdr:rowOff>
+      <xdr:rowOff>40291</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615167</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>172080</xdr:rowOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>11659</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -23063,7 +23073,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="175167" y="1885133"/>
+          <a:off x="175167" y="1911870"/>
           <a:ext cx="1440000" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -23229,7 +23239,19 @@
             <a:rPr sz="1400" b="1">
               <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>60%</a:t>
+            <a:t>6</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="1">
+              <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>1</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr sz="1400" b="1">
+              <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>%</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -23241,13 +23263,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>175167</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>137570</xdr:rowOff>
+      <xdr:rowOff>164307</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615167</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>108939</xdr:rowOff>
+      <xdr:rowOff>135676</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -23262,7 +23284,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="175167" y="4255044"/>
+          <a:off x="175167" y="4281781"/>
           <a:ext cx="1440000" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -23409,7 +23431,7 @@
               </a:solidFill>
               <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>40</a:t>
+            <a:t>39</a:t>
           </a:r>
           <a:r>
             <a:rPr sz="1400" b="1">
@@ -23430,13 +23452,13 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>382641</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>13554</xdr:rowOff>
+      <xdr:rowOff>40291</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>579378</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>172080</xdr:rowOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>11659</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -23451,8 +23473,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5616378" y="1885133"/>
-          <a:ext cx="1440000" cy="720000"/>
+          <a:off x="6050852" y="1911870"/>
+          <a:ext cx="1533579" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -23607,10 +23629,16 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
+            <a:rPr lang="en-US" sz="1400" b="1">
+              <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>5</a:t>
+          </a:r>
+          <a:r>
             <a:rPr sz="1400" b="1">
               <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>47%</a:t>
+            <a:t>7%</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -23622,13 +23650,13 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>382641</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>137570</xdr:rowOff>
+      <xdr:rowOff>164307</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>579378</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>108939</xdr:rowOff>
+      <xdr:rowOff>135676</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -23643,8 +23671,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5616378" y="4255044"/>
-          <a:ext cx="1440000" cy="720000"/>
+          <a:off x="6050852" y="4281781"/>
+          <a:ext cx="1533579" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -23802,13 +23830,22 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
+            <a:rPr lang="en-US" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>4</a:t>
+          </a:r>
+          <a:r>
             <a:rPr sz="1400" b="1">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:latin typeface="Arial Narrow" panose="020B0606020202030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>53%</a:t>
+            <a:t>3%</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -23820,13 +23857,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>796383</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>15594</xdr:rowOff>
+      <xdr:rowOff>42331</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>484172</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>174120</xdr:rowOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>13699</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -23841,8 +23878,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2674646" y="1887173"/>
-          <a:ext cx="1800000" cy="720000"/>
+          <a:off x="2841751" y="1913910"/>
+          <a:ext cx="1973789" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -24054,13 +24091,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>796383</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>38318</xdr:rowOff>
+      <xdr:rowOff>65055</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>484172</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>9686</xdr:rowOff>
+      <xdr:rowOff>36423</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -24075,8 +24112,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2674646" y="2845686"/>
-          <a:ext cx="1800000" cy="720000"/>
+          <a:off x="2841751" y="2872423"/>
+          <a:ext cx="1973789" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -24258,13 +24295,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>796383</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>89885</xdr:rowOff>
+      <xdr:rowOff>116622</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>484172</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>61253</xdr:rowOff>
+      <xdr:rowOff>87990</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -24279,8 +24316,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2674646" y="4768832"/>
-          <a:ext cx="1800000" cy="720000"/>
+          <a:off x="2841751" y="4795569"/>
+          <a:ext cx="1973789" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -24438,13 +24475,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>804741</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>61041</xdr:rowOff>
+      <xdr:rowOff>87778</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>492530</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>32410</xdr:rowOff>
+      <xdr:rowOff>59147</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -24459,8 +24496,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2683004" y="3804199"/>
-          <a:ext cx="1800000" cy="720000"/>
+          <a:off x="2850109" y="3830936"/>
+          <a:ext cx="1973789" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -24641,14 +24678,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>796383</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>177988</xdr:rowOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>17568</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>484172</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>149357</xdr:rowOff>
+      <xdr:rowOff>176094</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -24663,8 +24700,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2674646" y="926620"/>
-          <a:ext cx="1800000" cy="720000"/>
+          <a:off x="2841751" y="953357"/>
+          <a:ext cx="1973789" cy="720000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -24837,13 +24874,13 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>300387</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>26737</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>99861</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>82365</xdr:rowOff>
+      <xdr:rowOff>109102</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -24858,8 +24895,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5534124" y="0"/>
-          <a:ext cx="2286000" cy="830997"/>
+          <a:off x="5968598" y="26737"/>
+          <a:ext cx="2473158" cy="830997"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -24986,13 +25023,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>594916</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>24205</xdr:rowOff>
+      <xdr:rowOff>50942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>147074</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>47506</xdr:rowOff>
+      <xdr:rowOff>74243</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -25007,8 +25044,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2473179" y="24205"/>
-          <a:ext cx="2286000" cy="584775"/>
+          <a:off x="2640284" y="50942"/>
+          <a:ext cx="2506579" cy="584775"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -25135,13 +25172,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615167</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>123255</xdr:rowOff>
+      <xdr:rowOff>149992</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>796383</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>75569</xdr:rowOff>
+      <xdr:rowOff>102306</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -25159,8 +25196,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1615167" y="4615044"/>
-          <a:ext cx="1059479" cy="513788"/>
+          <a:off x="1615167" y="4641781"/>
+          <a:ext cx="1226584" cy="513788"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst/>
@@ -25194,13 +25231,13 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>484172</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>123255</xdr:rowOff>
+      <xdr:rowOff>149992</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>382641</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>75569</xdr:rowOff>
+      <xdr:rowOff>102306</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -25219,8 +25256,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="4474646" y="4615044"/>
-          <a:ext cx="1141732" cy="513788"/>
+          <a:off x="4815540" y="4641781"/>
+          <a:ext cx="1235312" cy="513788"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst/>
@@ -25253,14 +25290,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615167</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>186396</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>25975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>796383</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>24002</xdr:rowOff>
+      <xdr:rowOff>50739</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -25279,8 +25316,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1615167" y="2245133"/>
-          <a:ext cx="1059479" cy="960553"/>
+          <a:off x="1615167" y="2271870"/>
+          <a:ext cx="1226584" cy="960553"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -25313,76 +25350,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>484172</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>24002</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>382641</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>123255</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="20" name="Connector: Curved 19">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6170145-26C0-46A5-2EEB-B126E2454FC7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:cxnSpLocks/>
-          <a:stCxn id="11" idx="3"/>
-          <a:endCxn id="9" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4474646" y="3205686"/>
-          <a:ext cx="1141732" cy="1409358"/>
-        </a:xfrm>
-        <a:prstGeom prst="curvedConnector3">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:solidFill>
-            <a:srgbClr val="49B958"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615167</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>46725</xdr:rowOff>
+      <xdr:rowOff>73462</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>804741</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>123255</xdr:rowOff>
+      <xdr:rowOff>149992</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -25401,8 +25378,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="1615167" y="4164199"/>
-          <a:ext cx="1067837" cy="450845"/>
+          <a:off x="1615167" y="4190936"/>
+          <a:ext cx="1234942" cy="450845"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -25437,14 +25414,14 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>492530</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>186396</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>25975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>382641</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>46725</xdr:rowOff>
+      <xdr:rowOff>73462</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -25463,8 +25440,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="4483004" y="2245133"/>
-          <a:ext cx="1133374" cy="1919066"/>
+          <a:off x="4823898" y="2271870"/>
+          <a:ext cx="1226954" cy="1919066"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -25499,14 +25476,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1615167</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>186396</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>25975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>796383</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>1278</xdr:rowOff>
+      <xdr:rowOff>28015</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -25525,8 +25502,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1615167" y="2245133"/>
-          <a:ext cx="1059479" cy="2040"/>
+          <a:off x="1615167" y="2271870"/>
+          <a:ext cx="1226584" cy="2040"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -25561,14 +25538,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>1623525</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>163673</xdr:rowOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>3252</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>804741</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>186396</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>25975</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -25585,8 +25562,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="1623525" y="1286620"/>
-          <a:ext cx="1059479" cy="958513"/>
+          <a:off x="1623525" y="1313357"/>
+          <a:ext cx="1226584" cy="958513"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -25621,14 +25598,14 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>484172</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>186396</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>25975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>382641</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>1278</xdr:rowOff>
+      <xdr:rowOff>28015</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -25647,70 +25624,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="4474646" y="2245133"/>
-          <a:ext cx="1141732" cy="2040"/>
-        </a:xfrm>
-        <a:prstGeom prst="curvedConnector3">
-          <a:avLst>
-            <a:gd name="adj1" fmla="val 50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:ln>
-          <a:solidFill>
-            <a:srgbClr val="448114"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>484172</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>163673</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>382641</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>186396</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="26" name="Connector: Curved 25">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0243F90-B5A1-13D1-F549-1C65A83C7B1A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:cxnSpLocks/>
-          <a:stCxn id="14" idx="3"/>
-          <a:endCxn id="8" idx="1"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4474646" y="1286620"/>
-          <a:ext cx="1141732" cy="958513"/>
+          <a:off x="4815540" y="2271870"/>
+          <a:ext cx="1235312" cy="2040"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -25748,23 +25663,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>387685</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>113631</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>374316</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>13369</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>163095</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>152399</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>336884</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>72190</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Graphic 7">
+        <xdr:cNvPr id="3" name="Graphic 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D62AFC39-77AE-2EC9-D20A-8B62D19B45BF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{716E5DC9-99BD-0BA3-C359-8E37FEEDDA8F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -25786,58 +25701,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4050632" y="1236578"/>
-          <a:ext cx="5791200" cy="4343400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>561474</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>32714</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>655051</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>106948</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Graphic 9">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68FC0C24-2E6C-E45B-6177-48FCC5176BF4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4892842" y="5647451"/>
-          <a:ext cx="4772525" cy="4753181"/>
+          <a:off x="3368842" y="2072106"/>
+          <a:ext cx="7315200" cy="5486400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -26456,15 +26321,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>508000</xdr:colOff>
+      <xdr:colOff>507999</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>101600</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>12700</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>516466</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -26493,8 +26358,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3251200" y="2400300"/>
-          <a:ext cx="4978400" cy="3733800"/>
+          <a:off x="3251199" y="2400300"/>
+          <a:ext cx="6739467" cy="5054600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -26711,10 +26576,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>575327</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>45357</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>175710</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -26744,7 +26609,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3784345" cy="5069114"/>
+          <a:ext cx="4592411" cy="6151514"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -26918,15 +26783,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>698500</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>444500</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -26955,8 +26820,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1803400" y="165100"/>
-          <a:ext cx="4660900" cy="4914900"/>
+          <a:off x="1130300" y="203200"/>
+          <a:ext cx="4660900" cy="5384800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -27185,22 +27050,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>468546</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>147961</xdr:rowOff>
+      <xdr:colOff>209611</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>258932</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>123301</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>496270</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>24661</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Graphic 3">
+        <xdr:cNvPr id="8" name="Graphic 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9430A13D-1709-3C9D-131B-508BAEC786E5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D868AAF-C6C3-BB49-9004-606597526659}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -27222,8 +27087,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1689226" y="1442621"/>
-          <a:ext cx="3070191" cy="3859321"/>
+          <a:off x="1430291" y="554854"/>
+          <a:ext cx="6476367" cy="6128059"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -27446,13 +27311,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>300817</xdr:colOff>
+      <xdr:colOff>300816</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>490151</xdr:colOff>
+      <xdr:colOff>647699</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>132018</xdr:rowOff>
     </xdr:to>
@@ -27788,10 +27653,10 @@
       <xdr:rowOff>19843</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>238125</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>3368</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>597928</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -27821,7 +27686,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10556875" y="813593"/>
-          <a:ext cx="5913438" cy="7921025"/>
+          <a:ext cx="6947928" cy="9306720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -35554,7 +35419,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>82</v>
       </c>
       <c r="B2" t="s">
@@ -35562,7 +35427,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="13" t="s">
         <v>83</v>
       </c>
       <c r="B3" t="s">
@@ -35570,7 +35435,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="14" t="s">
         <v>84</v>
       </c>
       <c r="B4" t="s">
@@ -35578,7 +35443,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="15" t="s">
         <v>85</v>
       </c>
       <c r="B5" t="s">
@@ -35586,7 +35451,7 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="16" t="s">
         <v>86</v>
       </c>
       <c r="B6" t="s">
@@ -35594,7 +35459,7 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="17" t="s">
         <v>87</v>
       </c>
       <c r="B7" t="s">
@@ -35602,7 +35467,7 @@
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="18" t="s">
         <v>88</v>
       </c>
       <c r="B8" t="s">
@@ -35610,7 +35475,7 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="19" t="s">
         <v>89</v>
       </c>
       <c r="B9" t="s">
@@ -35634,7 +35499,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE41FDF4-A516-4160-9446-E74F46A2311D}">
-  <dimension ref="A22:K50"/>
+  <dimension ref="A22:K54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
@@ -35876,34 +35741,56 @@
       <c r="H40" s="7"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B41" s="7"/>
       <c r="H41" s="7"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B42" s="7"/>
       <c r="H42" s="7"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B43" s="7"/>
       <c r="H43" s="7"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B44" s="7"/>
       <c r="H44" s="7"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B45" s="7"/>
       <c r="H45" s="7"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B46" s="7"/>
       <c r="H46" s="7"/>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B47" s="7"/>
       <c r="H47" s="7"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B48" s="7"/>
       <c r="H48" s="7"/>
     </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B49" s="7"/>
       <c r="H49" s="7"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B50" s="7"/>
       <c r="H50" s="7"/>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B51" s="7"/>
+    </row>
+    <row r="52" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B52" s="7"/>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B53" s="7"/>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B54" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -35996,7 +35883,7 @@
         <v>48</v>
       </c>
       <c r="B27" s="7">
-        <v>0.53</v>
+        <v>0.43</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -36012,7 +35899,7 @@
         <v>49</v>
       </c>
       <c r="B28" s="7">
-        <v>0.47</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -37009,7 +36896,7 @@
       <c r="C22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="23"/>
+      <c r="D22" s="21"/>
       <c r="E22" s="3" t="s">
         <v>65</v>
       </c>
@@ -37211,7 +37098,7 @@
       <c r="C29" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="23"/>
+      <c r="D29" s="21"/>
       <c r="E29" s="3" t="s">
         <v>65</v>
       </c>
@@ -37287,7 +37174,7 @@
       <c r="C32" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="23"/>
+      <c r="D32" s="21"/>
       <c r="E32" s="3" t="s">
         <v>65</v>
       </c>
@@ -38679,7 +38566,7 @@
       <c r="B22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C22" s="23"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="3" t="s">
         <v>65</v>
       </c>
@@ -38839,7 +38726,7 @@
       <c r="B29" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="23"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="3" t="s">
         <v>65</v>
       </c>
@@ -38897,7 +38784,7 @@
       <c r="B32" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="23"/>
+      <c r="C32" s="21"/>
       <c r="D32" s="3" t="s">
         <v>65</v>
       </c>
@@ -39867,7 +39754,7 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="22">
+      <c r="B2" s="20">
         <v>0.314</v>
       </c>
       <c r="C2" s="2"/>
@@ -39892,8 +39779,8 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="22">
-        <v>0.26700000000000002</v>
+      <c r="B3" s="20">
+        <v>0.26</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -39917,7 +39804,7 @@
       <c r="A4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="20">
         <v>0.23400000000000001</v>
       </c>
       <c r="C4" s="2"/>
@@ -39942,7 +39829,7 @@
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="20">
         <v>0.217</v>
       </c>
       <c r="C5" s="2"/>
@@ -39967,7 +39854,7 @@
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="20">
         <v>0.13300000000000001</v>
       </c>
       <c r="C6" s="2"/>
@@ -39992,7 +39879,7 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="20">
         <v>0.13200000000000001</v>
       </c>
       <c r="C7" s="2"/>
@@ -40017,7 +39904,7 @@
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="20">
         <v>0.122</v>
       </c>
       <c r="C8" s="2"/>
@@ -40042,7 +39929,7 @@
       <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="20">
         <v>9.1999999999999998E-2</v>
       </c>
       <c r="C9" s="2"/>
@@ -40067,7 +39954,7 @@
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="20">
         <v>9.0999999999999998E-2</v>
       </c>
       <c r="C10" s="2"/>
@@ -40092,7 +39979,7 @@
       <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="20">
         <v>8.8999999999999996E-2</v>
       </c>
       <c r="C11" s="2"/>
@@ -40117,7 +40004,7 @@
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="20">
         <v>6.5000000000000002E-2</v>
       </c>
       <c r="C12" s="2"/>
@@ -40142,7 +40029,7 @@
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="20">
         <v>1.4E-2</v>
       </c>
       <c r="C13" s="2"/>
@@ -40577,7 +40464,7 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="11">
         <v>0.314</v>
       </c>
       <c r="C2" s="2"/>
@@ -40602,7 +40489,7 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="11">
         <v>0.26700000000000002</v>
       </c>
       <c r="C3" s="2"/>
@@ -40627,7 +40514,7 @@
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="11">
         <v>0.23400000000000001</v>
       </c>
       <c r="C4" s="2"/>
@@ -40652,7 +40539,7 @@
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="11">
         <v>0.217</v>
       </c>
       <c r="C5" s="2"/>
@@ -40677,7 +40564,7 @@
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="11">
         <v>0.13300000000000001</v>
       </c>
       <c r="C6" s="2"/>
@@ -40702,7 +40589,7 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="11">
         <v>0.13200000000000001</v>
       </c>
       <c r="C7" s="2"/>
@@ -40727,7 +40614,7 @@
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="11">
         <v>0.122</v>
       </c>
       <c r="C8" s="2"/>
@@ -40752,7 +40639,7 @@
       <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="11">
         <v>9.1999999999999998E-2</v>
       </c>
       <c r="C9" s="2"/>
@@ -40777,7 +40664,7 @@
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="11">
         <v>9.0999999999999998E-2</v>
       </c>
       <c r="C10" s="2"/>
@@ -40802,7 +40689,7 @@
       <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="11">
         <v>8.8999999999999996E-2</v>
       </c>
       <c r="C11" s="2"/>
@@ -40827,7 +40714,7 @@
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="11">
         <v>6.5000000000000002E-2</v>
       </c>
       <c r="C12" s="2"/>
@@ -40852,7 +40739,7 @@
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="11">
         <v>1.4E-2</v>
       </c>
       <c r="C13" s="2"/>
@@ -41733,7 +41620,7 @@
       <c r="D22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="23" t="s">
+      <c r="E22" s="21" t="s">
         <v>16</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -41775,7 +41662,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="7">
-        <v>0.51</v>
+        <v>0.59</v>
       </c>
       <c r="F23" s="1">
         <v>0.57999999999999996</v>
@@ -41805,7 +41692,7 @@
         <v>26</v>
       </c>
       <c r="E24" s="7">
-        <v>0.58799999999999997</v>
+        <v>0.65</v>
       </c>
       <c r="F24" s="1">
         <v>0.57999999999999996</v>
@@ -41835,7 +41722,7 @@
         <v>25</v>
       </c>
       <c r="E25" s="7">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="F25" s="1">
         <v>0.57999999999999996</v>
@@ -41865,7 +41752,7 @@
         <v>24</v>
       </c>
       <c r="E26" s="7">
-        <v>0.60099999999999998</v>
+        <v>0.6</v>
       </c>
       <c r="F26" s="1">
         <v>0.57999999999999996</v>
@@ -41890,7 +41777,7 @@
         <v>23</v>
       </c>
       <c r="E27" s="7">
-        <v>0.66</v>
+        <v>0.59</v>
       </c>
       <c r="F27" s="1">
         <v>0.57999999999999996</v>
@@ -41913,7 +41800,7 @@
         <v>22</v>
       </c>
       <c r="E28" s="7">
-        <v>0.60099999999999998</v>
+        <v>0.51</v>
       </c>
       <c r="F28" s="1">
         <v>0.57999999999999996</v>
@@ -41938,7 +41825,7 @@
       <c r="D29" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="23" t="s">
+      <c r="E29" s="21" t="s">
         <v>16</v>
       </c>
       <c r="F29" s="3" t="s">
@@ -41988,7 +41875,7 @@
         <v>30</v>
       </c>
       <c r="E31" s="7">
-        <v>0.72</v>
+        <v>0.7</v>
       </c>
       <c r="F31" s="1">
         <v>0.57999999999999996</v>
@@ -42013,7 +41900,7 @@
       <c r="D32" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="23" t="s">
+      <c r="E32" s="21" t="s">
         <v>16</v>
       </c>
       <c r="F32" s="3" t="s">
@@ -42126,6 +42013,12 @@
       <c r="R38" s="2"/>
     </row>
     <row r="39" spans="3:18" x14ac:dyDescent="0.2">
+      <c r="F39" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
@@ -42139,84 +42032,144 @@
     <row r="40" spans="3:18" x14ac:dyDescent="0.2">
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
-      <c r="F40" s="6"/>
-      <c r="G40" s="3"/>
+      <c r="F40" t="s">
+        <v>18</v>
+      </c>
+      <c r="G40" s="7">
+        <v>0.56399999999999995</v>
+      </c>
       <c r="H40" s="3"/>
     </row>
     <row r="41" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="F41" s="7"/>
-      <c r="G41" s="1"/>
+      <c r="F41" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="7">
+        <v>0.60299999999999998</v>
+      </c>
       <c r="H41" s="1"/>
     </row>
     <row r="42" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="F42" s="7"/>
-      <c r="G42" s="1"/>
+      <c r="F42" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="H42" s="1"/>
     </row>
     <row r="43" spans="3:18" x14ac:dyDescent="0.2">
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
-      <c r="F43" s="6"/>
-      <c r="G43" s="3"/>
+      <c r="F43" t="s">
+        <v>22</v>
+      </c>
+      <c r="G43" s="7">
+        <v>0.51</v>
+      </c>
       <c r="H43" s="3"/>
     </row>
     <row r="44" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="F44" s="7"/>
-      <c r="G44" s="1"/>
+      <c r="F44" t="s">
+        <v>23</v>
+      </c>
+      <c r="G44" s="7">
+        <v>0.58799999999999997</v>
+      </c>
       <c r="H44" s="1"/>
     </row>
     <row r="45" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="F45" s="7"/>
-      <c r="G45" s="1"/>
+      <c r="F45" t="s">
+        <v>24</v>
+      </c>
+      <c r="G45" s="7">
+        <v>0.6</v>
+      </c>
       <c r="H45" s="1"/>
     </row>
     <row r="46" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="F46" s="7"/>
-      <c r="G46" s="1"/>
+      <c r="F46" t="s">
+        <v>25</v>
+      </c>
+      <c r="G46" s="7">
+        <v>0.59</v>
+      </c>
       <c r="H46" s="1"/>
     </row>
     <row r="47" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="F47" s="7"/>
-      <c r="G47" s="1"/>
+      <c r="F47" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="7">
+        <v>0.65</v>
+      </c>
       <c r="H47" s="1"/>
     </row>
     <row r="48" spans="3:18" x14ac:dyDescent="0.2">
-      <c r="F48" s="7"/>
-      <c r="G48" s="1"/>
+      <c r="F48" t="s">
+        <v>27</v>
+      </c>
+      <c r="G48" s="7">
+        <v>0.59</v>
+      </c>
       <c r="H48" s="1"/>
     </row>
     <row r="49" spans="4:8" x14ac:dyDescent="0.2">
-      <c r="F49" s="7"/>
-      <c r="G49" s="1"/>
+      <c r="F49" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="H49" s="1"/>
     </row>
     <row r="50" spans="4:8" x14ac:dyDescent="0.2">
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
-      <c r="F50" s="6"/>
-      <c r="G50" s="3"/>
+      <c r="F50" t="s">
+        <v>29</v>
+      </c>
+      <c r="G50" s="7">
+        <v>0.53400000000000003</v>
+      </c>
       <c r="H50" s="3"/>
     </row>
     <row r="51" spans="4:8" x14ac:dyDescent="0.2">
-      <c r="F51" s="7"/>
-      <c r="G51" s="1"/>
+      <c r="F51" t="s">
+        <v>30</v>
+      </c>
+      <c r="G51" s="7">
+        <v>0.7</v>
+      </c>
       <c r="H51" s="1"/>
     </row>
     <row r="52" spans="4:8" x14ac:dyDescent="0.2">
-      <c r="F52" s="7"/>
-      <c r="G52" s="1"/>
+      <c r="F52" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="H52" s="1"/>
     </row>
     <row r="53" spans="4:8" x14ac:dyDescent="0.2">
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
-      <c r="F53" s="6"/>
-      <c r="G53" s="3"/>
+      <c r="F53" t="s">
+        <v>32</v>
+      </c>
+      <c r="G53" s="7">
+        <v>0.58199999999999996</v>
+      </c>
       <c r="H53" s="3"/>
     </row>
     <row r="54" spans="4:8" x14ac:dyDescent="0.2">
-      <c r="F54" s="7"/>
-      <c r="G54" s="1"/>
+      <c r="F54" t="s">
+        <v>33</v>
+      </c>
+      <c r="G54" s="7">
+        <v>0.58399999999999996</v>
+      </c>
       <c r="H54" s="1"/>
     </row>
     <row r="55" spans="4:8" x14ac:dyDescent="0.2">
@@ -42652,7 +42605,7 @@
         <v>25</v>
       </c>
       <c r="H26" s="7">
-        <v>0.60099999999999998</v>
+        <v>0.59</v>
       </c>
       <c r="I26" s="1">
         <v>0.58299999999999996</v>
@@ -42677,7 +42630,7 @@
         <v>26</v>
       </c>
       <c r="H27" s="7">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="I27" s="1">
         <v>0.58299999999999996</v>
@@ -42691,7 +42644,7 @@
         <v>27</v>
       </c>
       <c r="H28" s="7">
-        <v>0.60099999999999998</v>
+        <v>0.59</v>
       </c>
       <c r="I28" s="1">
         <v>0.58299999999999996</v>
@@ -42739,7 +42692,7 @@
         <v>30</v>
       </c>
       <c r="H31" s="7">
-        <v>0.72199999999999998</v>
+        <v>0.7</v>
       </c>
       <c r="I31" s="1">
         <v>0.58299999999999996</v>
@@ -43190,11 +43143,11 @@
       <c r="C20" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="11">
-        <v>4</v>
+      <c r="D20" s="10">
+        <v>3.7</v>
       </c>
       <c r="E20">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="2"/>
@@ -43223,10 +43176,10 @@
         <v>19</v>
       </c>
       <c r="D21" s="10">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="E21">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="2"/>
@@ -43257,7 +43210,7 @@
       <c r="C22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="6"/>
+      <c r="D22" s="22"/>
       <c r="E22" s="3" t="s">
         <v>76</v>
       </c>
@@ -43287,11 +43240,11 @@
       <c r="C23" t="s">
         <v>27</v>
       </c>
-      <c r="D23">
-        <v>5.3</v>
+      <c r="D23" s="23">
+        <v>5</v>
       </c>
       <c r="E23">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="2"/>
@@ -43316,11 +43269,11 @@
       <c r="C24" t="s">
         <v>26</v>
       </c>
-      <c r="D24">
-        <v>5.3</v>
+      <c r="D24" s="23">
+        <v>4.5999999999999996</v>
       </c>
       <c r="E24">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="2"/>
@@ -43345,11 +43298,11 @@
       <c r="C25" t="s">
         <v>25</v>
       </c>
-      <c r="D25">
-        <v>4.8</v>
+      <c r="D25" s="23">
+        <v>4.4000000000000004</v>
       </c>
       <c r="E25">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="2"/>
@@ -43374,11 +43327,11 @@
       <c r="C26" t="s">
         <v>24</v>
       </c>
-      <c r="D26">
-        <v>4.4000000000000004</v>
+      <c r="D26" s="23">
+        <v>4</v>
       </c>
       <c r="E26">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="2"/>
@@ -43403,11 +43356,11 @@
       <c r="C27" t="s">
         <v>23</v>
       </c>
-      <c r="D27">
-        <v>3.3</v>
+      <c r="D27" s="23">
+        <v>3.2</v>
       </c>
       <c r="E27">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="2"/>
@@ -43426,11 +43379,11 @@
       <c r="C28" t="s">
         <v>22</v>
       </c>
-      <c r="D28">
-        <v>3.1</v>
+      <c r="D28" s="23">
+        <v>3</v>
       </c>
       <c r="E28">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="2"/>
@@ -43452,7 +43405,7 @@
       <c r="C29" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="6"/>
+      <c r="D29" s="22"/>
       <c r="E29" s="3" t="s">
         <v>76</v>
       </c>
@@ -43476,11 +43429,11 @@
       <c r="C30" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="12">
-        <v>3.4</v>
-      </c>
-      <c r="E30" s="12">
-        <v>4.0999999999999996</v>
+      <c r="D30" s="23">
+        <v>3.3</v>
+      </c>
+      <c r="E30">
+        <v>3.8</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="2"/>
@@ -43499,11 +43452,11 @@
       <c r="C31" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="12">
-        <v>5.7</v>
-      </c>
-      <c r="E31" s="12">
-        <v>4.0999999999999996</v>
+      <c r="D31" s="23">
+        <v>5</v>
+      </c>
+      <c r="E31">
+        <v>3.8</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="2"/>
@@ -43525,7 +43478,7 @@
       <c r="C32" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="6"/>
+      <c r="D32" s="22"/>
       <c r="E32" s="3" t="s">
         <v>76</v>
       </c>
@@ -43549,11 +43502,11 @@
       <c r="C33" t="s">
         <v>32</v>
       </c>
-      <c r="D33">
-        <v>4.0999999999999996</v>
+      <c r="D33" s="23">
+        <v>3.8</v>
       </c>
       <c r="E33">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="2"/>
@@ -43572,11 +43525,11 @@
       <c r="C34" t="s">
         <v>33</v>
       </c>
-      <c r="D34">
-        <v>4.2</v>
+      <c r="D34" s="23">
+        <v>4</v>
       </c>
       <c r="E34">
-        <v>4.0999999999999996</v>
+        <v>3.8</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="2"/>
@@ -47917,26 +47870,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="46f3a809-46a3-44ee-a0f1-42a271529c86">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="69276225-f05c-44c5-92dc-c999460a4149" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006BF094976B1C6245BAB5BCECAC284645" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="347dc9eaee87b4cbb901bc584e0b214d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="69276225-f05c-44c5-92dc-c999460a4149" xmlns:ns3="46f3a809-46a3-44ee-a0f1-42a271529c86" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="32796ae3933d308c0b8b72e1382e1089" ns2:_="" ns3:_="">
     <xsd:import namespace="69276225-f05c-44c5-92dc-c999460a4149"/>
@@ -48185,32 +48118,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{477416C7-F190-4CB3-9882-326CCF62513A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="46f3a809-46a3-44ee-a0f1-42a271529c86">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="69276225-f05c-44c5-92dc-c999460a4149" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B93DCC44-58EE-4CE6-9895-20B9272F964D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="46f3a809-46a3-44ee-a0f1-42a271529c86"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="69276225-f05c-44c5-92dc-c999460a4149"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7901C35-45A5-467C-928A-FE6D7B392357}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -48227,4 +48155,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B93DCC44-58EE-4CE6-9895-20B9272F964D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="69276225-f05c-44c5-92dc-c999460a4149"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="46f3a809-46a3-44ee-a0f1-42a271529c86"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{477416C7-F190-4CB3-9882-326CCF62513A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>